<commit_message>
docs: Research MySQL Optimization & RelationalDB_Internal
</commit_message>
<xml_diff>
--- a/Progress.xlsx
+++ b/Progress.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\QuintetCompany\projects\mini_dbms\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\QuintetCompany\projects\mini_dbms\mini_dbms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{490A82BB-DE9E-436B-8FF4-14A1A2A5260E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B92AE8B-C976-4818-AA39-44B5361A4EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="8" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overall" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="684">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="813" uniqueCount="696">
   <si>
     <t xml:space="preserve">Tôi muốn làm ra một hệ thống DBMS dựa trên kiến trúc và thuật toán của MySQL.
 Lí do thực hiện dự án, trong quá trình làm việc phát triển các ứng dụng và sử dụng MySQL tôi gặp vấn đề trong việc tối ưu truy vấn để giảm thiểu thời gian thực thi của một câu truy vấn. Tôi đã làm tìm hiểu cách tối ưu thì tôi biết được có cách là dùng index và cũng đã tìm hiểu về execution plan để hiểu khi DBMS thực thi một câu query thì cần làm những bước nào. Tuy nhiên tôi chưa thể hiểu rõ được khi nào thì dùng index và khi nào không nên và ngoài ra còn những cách nào khác không.
@@ -9948,6 +9948,850 @@
       <t>DDL hoặc thành công hoàn toàn, hoặc rollback hoàn toàn.</t>
     </r>
   </si>
+  <si>
+    <t>Q023</t>
+  </si>
+  <si>
+    <t>NDB Cluster là gì?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NDB Cluster là gì?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+thường gọi đầy đủ là MySQL NDB Cluster
+là một </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>kiến trúc cơ sở dữ liệu phân tán (distributed database)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> được thiết kế cho </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>high availability (HA) và horizontal scalability</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+trong đó </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>dữ liệu được chia nhỏ (sharding) và nhân bản (replication) trên nhiều node in-memory.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Tồn tại trong hệ sinh thái MySQL, dưới dạng 
+                </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>storage engine NDB + kiến trúc cluster riêng</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Phù hợp:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Telecom (HLR/HSS), Real-time OLTP, 99.999% uptime, Write-heavy + latency thấp
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Không phù hợp:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> OLAP, JOIN phức tạp, Dataset quá lớn (RAM hạn chế), SQL linh hoạt (NDB hạn chế optimizer)
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Kiến trúc của NDB Cluster gồm 3 loại node chính</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1. SQL Node:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Chạy MySQL Server (mysqld), nhận query SQL
+    SQL Node không lưu dữ liệu
+ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2. Data Node:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Lưu dữ liệu bằng NDB engine (RAM + disk)
+    Data Node không parse SQL
+ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3. Management Node:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Quản lý cấu hình, startup, giám sát cluster
+    Mọi thứ giao tiếp qua NDB API
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Cách NDB Cluster lưu dữ liệu:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+ 1. Dữ liệu được partition theo primary key
+ 2. Mỗi partition được replicate sang nhiều Data Node
+ 3. Truy cập chủ yếu in-memory
+ 4. Disk dùng cho redo log / checkpoint, không phải primary access path
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Ưu điểm: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+ 1. Fail node không mất dữ liệu
+ 2. Scale bằng cách thêm Data Node
+ 3. Độ trễ cực thấp cho OLTP</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NDB = Network DataBase</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+ - Dữ liệu không nằm cục bộ trong mysqld
+ - Dữ liệu được truy cập qua network tới data node
+ - Mọi thao tác CRUD đều đi qua NDB API → RPC / message passing
+ - Kiến trúc shared-nothing, distributed
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Lịch sử:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+NDB được phát triển bởi công ty MySQL AB
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Mục tiêu ban đầu:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Telecom-grade database, High Availability, Real-time processing
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Đặc điểm của NDB liên quan đến "Network"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1. SQL node ↔ Data node:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> TCP/IP
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2. Transaction:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Distributed transaction
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3. Locking:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Distributed locking
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4. Logging:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Distributed redo
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>5. Failover:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Node-to-node</t>
+    </r>
+  </si>
+  <si>
+    <t>Sargable conditions là gì?</t>
+  </si>
+  <si>
+    <t>Index Eligibility là gì?</t>
+  </si>
+  <si>
+    <t>Q024</t>
+  </si>
+  <si>
+    <t>Q025</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Ví dụ:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Sargable</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+WHERE age = 18
+WHERE age &gt; 18
+WHERE age BETWEEN 18 AND 25
+WHERE created_at &gt;= '2025-01-01'
+=&gt; MySQL:
+ - Biết bắt đầu từ đâu
+ - Biết dừng ở đâu trong B-tree index
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Not sargable</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+WHERE YEAR(created_at) = 2025
+WHERE age + 1 = 18
+WHERE UPPER(name) = 'JOHN'
+WHERE price * 2 &gt; 100
+=&gt; MySQL:
+ - Phải tính toán cho từng row
+ - Không dùng index
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Sargable = Search ARGument ABLE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Một điều kiện WHERE được gọi là sargable</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> nếu </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MySQL có thể dùng nó</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> để thực hiện </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>index lookup</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> hoặc </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>index range scan</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quy tắc của Sargable:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Column phải đứng một mình:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> [</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>column</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="5"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>operator</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="3"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">constant]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Không được:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+ - Column nằm trong function
+ - Column nằm trong biểu thức toán học
+ - Column bị ép kiểu ngầm (implicit cast)</t>
+    </r>
+  </si>
+  <si>
+    <t>Điều kiện             Is Sargable                       Lý do
+col = 5                        v                           Direct lookup
+col &gt; 5                        v                           Range scan
+col IN (1,2,3)              v                           Multiple lookups
+col LIKE 'abc%'           v                           Prefix range
+col LIKE '%abc'           x                           Không có start point
+FUNC(col) = x             x                           Index không áp dụng
+col + 1 = x                   x                           Expression trên col</t>
+  </si>
 </sst>
 </file>
 
@@ -9957,7 +10801,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -10133,6 +10977,22 @@
       <i/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="5"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="3"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -10713,7 +11573,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="210">
+  <cellXfs count="212">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -11136,6 +11996,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -11232,6 +12101,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -11239,15 +12117,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -11318,9 +12187,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -11451,7 +12317,7 @@
       <xdr:col>5</xdr:col>
       <xdr:colOff>800099</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>20634</xdr:rowOff>
+      <xdr:rowOff>16824</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -11851,7 +12717,7 @@
         <v>31</v>
       </c>
       <c r="F5" s="68"/>
-      <c r="G5" s="209" t="s">
+      <c r="G5" s="148" t="s">
         <v>91</v>
       </c>
     </row>
@@ -12010,10 +12876,10 @@
       </c>
     </row>
     <row r="8" spans="2:6" ht="171.6" x14ac:dyDescent="0.3">
-      <c r="B8" s="164" t="s">
+      <c r="B8" s="167" t="s">
         <v>104</v>
       </c>
-      <c r="C8" s="196" t="s">
+      <c r="C8" s="199" t="s">
         <v>233</v>
       </c>
       <c r="D8" s="13" t="s">
@@ -12021,36 +12887,36 @@
       </c>
     </row>
     <row r="9" spans="2:6" ht="78" x14ac:dyDescent="0.3">
-      <c r="B9" s="169"/>
-      <c r="C9" s="197"/>
+      <c r="B9" s="172"/>
+      <c r="C9" s="200"/>
       <c r="D9" s="13" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="10" spans="2:6" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B10" s="169"/>
-      <c r="C10" s="197"/>
+      <c r="B10" s="172"/>
+      <c r="C10" s="200"/>
       <c r="D10" s="13" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="11" spans="2:6" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="B11" s="169"/>
-      <c r="C11" s="197"/>
+      <c r="B11" s="172"/>
+      <c r="C11" s="200"/>
       <c r="D11" s="13" t="s">
         <v>237</v>
       </c>
     </row>
     <row r="12" spans="2:6" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B12" s="169"/>
-      <c r="C12" s="197"/>
+      <c r="B12" s="172"/>
+      <c r="C12" s="200"/>
       <c r="D12" s="13" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="13" spans="2:6" ht="78" x14ac:dyDescent="0.3">
-      <c r="B13" s="165"/>
-      <c r="C13" s="198"/>
+      <c r="B13" s="168"/>
+      <c r="C13" s="201"/>
       <c r="D13" s="13" t="s">
         <v>239</v>
       </c>
@@ -12065,7 +12931,7 @@
       <c r="D14" s="13" t="s">
         <v>243</v>
       </c>
-      <c r="E14" s="175" t="s">
+      <c r="E14" s="178" t="s">
         <v>249</v>
       </c>
     </row>
@@ -12079,7 +12945,7 @@
       <c r="D15" s="13" t="s">
         <v>244</v>
       </c>
-      <c r="E15" s="147"/>
+      <c r="E15" s="150"/>
       <c r="F15" s="105" t="s">
         <v>250</v>
       </c>
@@ -12094,7 +12960,7 @@
       <c r="D16" s="13" t="s">
         <v>245</v>
       </c>
-      <c r="E16" s="147"/>
+      <c r="E16" s="150"/>
     </row>
     <row r="17" spans="2:9" ht="280.8" x14ac:dyDescent="0.3">
       <c r="B17" s="103" t="s">
@@ -12111,10 +12977,10 @@
       </c>
     </row>
     <row r="18" spans="2:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="B18" s="164" t="s">
+      <c r="B18" s="167" t="s">
         <v>126</v>
       </c>
-      <c r="C18" s="196" t="s">
+      <c r="C18" s="199" t="s">
         <v>251</v>
       </c>
       <c r="D18" s="13" t="s">
@@ -12122,36 +12988,36 @@
       </c>
     </row>
     <row r="19" spans="2:9" ht="124.8" x14ac:dyDescent="0.3">
-      <c r="B19" s="169"/>
-      <c r="C19" s="197"/>
+      <c r="B19" s="172"/>
+      <c r="C19" s="200"/>
       <c r="D19" s="13" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="20" spans="2:9" ht="156" x14ac:dyDescent="0.3">
-      <c r="B20" s="169"/>
-      <c r="C20" s="197"/>
+      <c r="B20" s="172"/>
+      <c r="C20" s="200"/>
       <c r="D20" s="13" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="21" spans="2:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="B21" s="169"/>
-      <c r="C21" s="197"/>
+      <c r="B21" s="172"/>
+      <c r="C21" s="200"/>
       <c r="D21" s="13" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="22" spans="2:9" ht="140.4" x14ac:dyDescent="0.3">
-      <c r="B22" s="169"/>
-      <c r="C22" s="197"/>
+      <c r="B22" s="172"/>
+      <c r="C22" s="200"/>
       <c r="D22" s="13" t="s">
         <v>256</v>
       </c>
     </row>
     <row r="23" spans="2:9" ht="124.8" x14ac:dyDescent="0.3">
-      <c r="B23" s="165"/>
-      <c r="C23" s="198"/>
+      <c r="B23" s="168"/>
+      <c r="C23" s="201"/>
       <c r="D23" s="13" t="s">
         <v>257</v>
       </c>
@@ -12166,17 +13032,17 @@
       <c r="D24" s="106" t="s">
         <v>259</v>
       </c>
-      <c r="E24" s="193" t="s">
+      <c r="E24" s="196" t="s">
         <v>261</v>
       </c>
-      <c r="F24" s="194"/>
-      <c r="G24" s="195"/>
+      <c r="F24" s="197"/>
+      <c r="G24" s="198"/>
     </row>
     <row r="25" spans="2:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="H25" s="191" t="s">
+      <c r="H25" s="194" t="s">
         <v>260</v>
       </c>
-      <c r="I25" s="192"/>
+      <c r="I25" s="195"/>
     </row>
     <row r="26" spans="2:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="H26" s="107" t="s">
@@ -12234,7 +13100,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="33" spans="8:9" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="8:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="H33" s="107" t="s">
         <v>275</v>
       </c>
@@ -12485,8 +13351,8 @@
       </c>
     </row>
     <row r="3" spans="2:13" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B3" s="203"/>
-      <c r="C3" s="200" t="s">
+      <c r="B3" s="206"/>
+      <c r="C3" s="203" t="s">
         <v>677</v>
       </c>
       <c r="D3" s="146" t="s">
@@ -12494,36 +13360,36 @@
       </c>
     </row>
     <row r="4" spans="2:13" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B4" s="204"/>
-      <c r="C4" s="201"/>
+      <c r="B4" s="207"/>
+      <c r="C4" s="204"/>
       <c r="D4" s="146" t="s">
         <v>679</v>
       </c>
     </row>
     <row r="5" spans="2:13" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="B5" s="204"/>
-      <c r="C5" s="201"/>
+      <c r="B5" s="207"/>
+      <c r="C5" s="204"/>
       <c r="D5" s="146" t="s">
         <v>680</v>
       </c>
     </row>
     <row r="6" spans="2:13" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B6" s="204"/>
-      <c r="C6" s="201"/>
+      <c r="B6" s="207"/>
+      <c r="C6" s="204"/>
       <c r="D6" s="146" t="s">
         <v>681</v>
       </c>
     </row>
     <row r="7" spans="2:13" ht="78" x14ac:dyDescent="0.3">
-      <c r="B7" s="204"/>
-      <c r="C7" s="201"/>
+      <c r="B7" s="207"/>
+      <c r="C7" s="204"/>
       <c r="D7" s="146" t="s">
         <v>682</v>
       </c>
     </row>
     <row r="8" spans="2:13" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B8" s="205"/>
-      <c r="C8" s="202"/>
+      <c r="B8" s="208"/>
+      <c r="C8" s="205"/>
       <c r="D8" s="146" t="s">
         <v>683</v>
       </c>
@@ -12613,8 +13479,8 @@
       <c r="E17" s="117"/>
       <c r="F17" s="117"/>
       <c r="G17" s="117"/>
-      <c r="H17" s="199"/>
-      <c r="I17" s="199"/>
+      <c r="H17" s="202"/>
+      <c r="I17" s="202"/>
       <c r="J17" s="116"/>
       <c r="K17" s="116"/>
       <c r="L17" s="116"/>
@@ -13036,8 +13902,8 @@
       <c r="E11" s="117"/>
       <c r="F11" s="117"/>
       <c r="G11" s="117"/>
-      <c r="H11" s="199"/>
-      <c r="I11" s="199"/>
+      <c r="H11" s="202"/>
+      <c r="I11" s="202"/>
       <c r="J11" s="116"/>
       <c r="K11" s="116"/>
       <c r="L11" s="116"/>
@@ -13614,7 +14480,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE05D77F-849A-4AF5-8176-FA4DE5D23136}">
-  <dimension ref="B2:H54"/>
+  <dimension ref="B2:H57"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="94"/>
@@ -13815,10 +14681,10 @@
       <c r="E16" s="97"/>
     </row>
     <row r="17" spans="2:6" ht="120" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="164" t="s">
+      <c r="B17" s="167" t="s">
         <v>186</v>
       </c>
-      <c r="C17" s="153" t="s">
+      <c r="C17" s="156" t="s">
         <v>335</v>
       </c>
       <c r="D17" s="83" t="s">
@@ -13827,18 +14693,18 @@
       <c r="E17" s="97"/>
     </row>
     <row r="18" spans="2:6" ht="409.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="165"/>
-      <c r="C18" s="155"/>
+      <c r="B18" s="168"/>
+      <c r="C18" s="158"/>
       <c r="D18" s="13" t="s">
         <v>347</v>
       </c>
       <c r="E18" s="97"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="164" t="s">
+      <c r="B19" s="167" t="s">
         <v>187</v>
       </c>
-      <c r="C19" s="153" t="s">
+      <c r="C19" s="156" t="s">
         <v>348</v>
       </c>
       <c r="D19" s="123"/>
@@ -13850,8 +14716,8 @@
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="169"/>
-      <c r="C20" s="154"/>
+      <c r="B20" s="172"/>
+      <c r="C20" s="157"/>
       <c r="D20" s="128" t="s">
         <v>349</v>
       </c>
@@ -13863,8 +14729,8 @@
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="169"/>
-      <c r="C21" s="154"/>
+      <c r="B21" s="172"/>
+      <c r="C21" s="157"/>
       <c r="D21" s="128" t="s">
         <v>353</v>
       </c>
@@ -13876,8 +14742,8 @@
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="169"/>
-      <c r="C22" s="154"/>
+      <c r="B22" s="172"/>
+      <c r="C22" s="157"/>
       <c r="D22" s="128" t="s">
         <v>356</v>
       </c>
@@ -13889,8 +14755,8 @@
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="169"/>
-      <c r="C23" s="154"/>
+      <c r="B23" s="172"/>
+      <c r="C23" s="157"/>
       <c r="D23" s="128" t="s">
         <v>357</v>
       </c>
@@ -13902,8 +14768,8 @@
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B24" s="169"/>
-      <c r="C24" s="154"/>
+      <c r="B24" s="172"/>
+      <c r="C24" s="157"/>
       <c r="D24" s="128" t="s">
         <v>358</v>
       </c>
@@ -13915,8 +14781,8 @@
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B25" s="169"/>
-      <c r="C25" s="154"/>
+      <c r="B25" s="172"/>
+      <c r="C25" s="157"/>
       <c r="D25" s="128" t="s">
         <v>359</v>
       </c>
@@ -13928,8 +14794,8 @@
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B26" s="169"/>
-      <c r="C26" s="154"/>
+      <c r="B26" s="172"/>
+      <c r="C26" s="157"/>
       <c r="D26" s="128" t="s">
         <v>360</v>
       </c>
@@ -13941,8 +14807,8 @@
       </c>
     </row>
     <row r="27" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="169"/>
-      <c r="C27" s="154"/>
+      <c r="B27" s="172"/>
+      <c r="C27" s="157"/>
       <c r="D27" s="128" t="s">
         <v>361</v>
       </c>
@@ -13954,8 +14820,8 @@
       </c>
     </row>
     <row r="28" spans="2:6" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="169"/>
-      <c r="C28" s="154"/>
+      <c r="B28" s="172"/>
+      <c r="C28" s="157"/>
       <c r="D28" s="124" t="s">
         <v>373</v>
       </c>
@@ -13967,8 +14833,8 @@
       </c>
     </row>
     <row r="29" spans="2:6" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="169"/>
-      <c r="C29" s="154"/>
+      <c r="B29" s="172"/>
+      <c r="C29" s="157"/>
       <c r="D29" s="124" t="s">
         <v>374</v>
       </c>
@@ -13978,8 +14844,8 @@
       <c r="F29" s="110"/>
     </row>
     <row r="30" spans="2:6" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B30" s="169"/>
-      <c r="C30" s="154"/>
+      <c r="B30" s="172"/>
+      <c r="C30" s="157"/>
       <c r="D30" s="134" t="s">
         <v>394</v>
       </c>
@@ -13989,8 +14855,8 @@
       </c>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B31" s="169"/>
-      <c r="C31" s="154"/>
+      <c r="B31" s="172"/>
+      <c r="C31" s="157"/>
       <c r="D31" s="128" t="s">
         <v>380</v>
       </c>
@@ -14002,8 +14868,8 @@
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B32" s="169"/>
-      <c r="C32" s="154"/>
+      <c r="B32" s="172"/>
+      <c r="C32" s="157"/>
       <c r="D32" s="128" t="s">
         <v>383</v>
       </c>
@@ -14015,8 +14881,8 @@
       </c>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B33" s="169"/>
-      <c r="C33" s="154"/>
+      <c r="B33" s="172"/>
+      <c r="C33" s="157"/>
       <c r="D33" s="128" t="s">
         <v>386</v>
       </c>
@@ -14028,8 +14894,8 @@
       </c>
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B34" s="169"/>
-      <c r="C34" s="154"/>
+      <c r="B34" s="172"/>
+      <c r="C34" s="157"/>
       <c r="D34" s="128" t="s">
         <v>389</v>
       </c>
@@ -14041,8 +14907,8 @@
       </c>
     </row>
     <row r="35" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B35" s="169"/>
-      <c r="C35" s="154"/>
+      <c r="B35" s="172"/>
+      <c r="C35" s="157"/>
       <c r="D35" s="134" t="s">
         <v>393</v>
       </c>
@@ -14052,8 +14918,8 @@
       </c>
     </row>
     <row r="36" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B36" s="169"/>
-      <c r="C36" s="154"/>
+      <c r="B36" s="172"/>
+      <c r="C36" s="157"/>
       <c r="D36" s="129" t="s">
         <v>395</v>
       </c>
@@ -14065,8 +14931,8 @@
       </c>
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B37" s="169"/>
-      <c r="C37" s="154"/>
+      <c r="B37" s="172"/>
+      <c r="C37" s="157"/>
       <c r="D37" s="133" t="s">
         <v>398</v>
       </c>
@@ -14074,8 +14940,8 @@
       <c r="F37" s="130"/>
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B38" s="169"/>
-      <c r="C38" s="154"/>
+      <c r="B38" s="172"/>
+      <c r="C38" s="157"/>
       <c r="D38" s="131" t="s">
         <v>399</v>
       </c>
@@ -14087,8 +14953,8 @@
       </c>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B39" s="169"/>
-      <c r="C39" s="154"/>
+      <c r="B39" s="172"/>
+      <c r="C39" s="157"/>
       <c r="D39" s="131" t="s">
         <v>400</v>
       </c>
@@ -14100,8 +14966,8 @@
       </c>
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B40" s="169"/>
-      <c r="C40" s="154"/>
+      <c r="B40" s="172"/>
+      <c r="C40" s="157"/>
       <c r="D40" s="131" t="s">
         <v>401</v>
       </c>
@@ -14113,8 +14979,8 @@
       </c>
     </row>
     <row r="41" spans="2:8" ht="78" x14ac:dyDescent="0.3">
-      <c r="B41" s="165"/>
-      <c r="C41" s="155"/>
+      <c r="B41" s="168"/>
+      <c r="C41" s="158"/>
       <c r="D41" s="135" t="s">
         <v>406</v>
       </c>
@@ -14125,7 +14991,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="42" spans="2:8" ht="390" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:8" ht="374.4" x14ac:dyDescent="0.3">
       <c r="B42" s="112" t="s">
         <v>188</v>
       </c>
@@ -14226,10 +15092,10 @@
       </c>
     </row>
     <row r="47" spans="2:8" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="B47" s="164" t="s">
+      <c r="B47" s="167" t="s">
         <v>193</v>
       </c>
-      <c r="C47" s="206" t="s">
+      <c r="C47" s="209" t="s">
         <v>645</v>
       </c>
       <c r="D47" s="83" t="s">
@@ -14239,8 +15105,8 @@
       <c r="F47" s="143"/>
     </row>
     <row r="48" spans="2:8" ht="220.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="169"/>
-      <c r="C48" s="207"/>
+      <c r="B48" s="172"/>
+      <c r="C48" s="210"/>
       <c r="D48" s="83" t="s">
         <v>656</v>
       </c>
@@ -14252,8 +15118,8 @@
       </c>
     </row>
     <row r="49" spans="2:6" ht="199.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="169"/>
-      <c r="C49" s="207"/>
+      <c r="B49" s="172"/>
+      <c r="C49" s="210"/>
       <c r="D49" s="83" t="s">
         <v>647</v>
       </c>
@@ -14265,8 +15131,8 @@
       </c>
     </row>
     <row r="50" spans="2:6" ht="250.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B50" s="169"/>
-      <c r="C50" s="207"/>
+      <c r="B50" s="172"/>
+      <c r="C50" s="210"/>
       <c r="D50" s="83" t="s">
         <v>648</v>
       </c>
@@ -14278,8 +15144,8 @@
       </c>
     </row>
     <row r="51" spans="2:6" ht="249.6" x14ac:dyDescent="0.3">
-      <c r="B51" s="169"/>
-      <c r="C51" s="207"/>
+      <c r="B51" s="172"/>
+      <c r="C51" s="210"/>
       <c r="D51" s="13" t="s">
         <v>649</v>
       </c>
@@ -14289,28 +15155,73 @@
       </c>
     </row>
     <row r="52" spans="2:6" ht="140.4" x14ac:dyDescent="0.3">
-      <c r="B52" s="169"/>
-      <c r="C52" s="207"/>
+      <c r="B52" s="172"/>
+      <c r="C52" s="210"/>
       <c r="D52" s="13" t="s">
         <v>650</v>
       </c>
       <c r="E52" s="97"/>
     </row>
     <row r="53" spans="2:6" ht="109.2" x14ac:dyDescent="0.3">
-      <c r="B53" s="169"/>
-      <c r="C53" s="207"/>
+      <c r="B53" s="172"/>
+      <c r="C53" s="210"/>
       <c r="D53" s="13" t="s">
         <v>651</v>
       </c>
       <c r="E53" s="97"/>
     </row>
     <row r="54" spans="2:6" ht="78" x14ac:dyDescent="0.3">
-      <c r="B54" s="165"/>
-      <c r="C54" s="208"/>
+      <c r="B54" s="168"/>
+      <c r="C54" s="211"/>
       <c r="D54" s="13" t="s">
         <v>652</v>
       </c>
       <c r="E54" s="97"/>
+    </row>
+    <row r="55" spans="2:6" ht="280.8" x14ac:dyDescent="0.3">
+      <c r="B55" s="95" t="s">
+        <v>684</v>
+      </c>
+      <c r="C55" s="13" t="s">
+        <v>685</v>
+      </c>
+      <c r="D55" s="83" t="s">
+        <v>686</v>
+      </c>
+      <c r="E55" s="13" t="s">
+        <v>687</v>
+      </c>
+      <c r="F55" s="147" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="56" spans="2:6" ht="280.8" x14ac:dyDescent="0.3">
+      <c r="B56" s="95" t="s">
+        <v>691</v>
+      </c>
+      <c r="C56" s="13" t="s">
+        <v>689</v>
+      </c>
+      <c r="D56" s="149" t="s">
+        <v>694</v>
+      </c>
+      <c r="E56" s="149" t="s">
+        <v>693</v>
+      </c>
+      <c r="F56" s="149" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="57" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B57" s="95" t="s">
+        <v>692</v>
+      </c>
+      <c r="C57" s="13" t="s">
+        <v>690</v>
+      </c>
+      <c r="D57" s="13"/>
+      <c r="E57" s="13"/>
+      <c r="F57" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -14424,10 +15335,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.4">
-      <c r="B2" s="150" t="s">
+      <c r="B2" s="153" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="150"/>
+      <c r="C2" s="153"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.4">
       <c r="C3" s="7" t="s">
@@ -14435,10 +15346,10 @@
       </c>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.4">
-      <c r="B4" s="150" t="s">
+      <c r="B4" s="153" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="150"/>
+      <c r="C4" s="153"/>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.4">
       <c r="C5" s="7" t="s">
@@ -14446,10 +15357,10 @@
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.4">
-      <c r="B6" s="150" t="s">
+      <c r="B6" s="153" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="150"/>
+      <c r="C6" s="153"/>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.4">
       <c r="C7" s="7" t="s">
@@ -14457,10 +15368,10 @@
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.4">
-      <c r="B8" s="150" t="s">
+      <c r="B8" s="153" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="150"/>
+      <c r="C8" s="153"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.4">
       <c r="C9" s="7" t="s">
@@ -14468,10 +15379,10 @@
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.4">
-      <c r="B10" s="150" t="s">
+      <c r="B10" s="153" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="150"/>
+      <c r="C10" s="153"/>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.4">
       <c r="D12" s="80" t="s">
@@ -14480,10 +15391,10 @@
     </row>
     <row r="13" spans="2:10" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D13" s="86"/>
-      <c r="E13" s="151" t="s">
+      <c r="E13" s="154" t="s">
         <v>334</v>
       </c>
-      <c r="F13" s="151"/>
+      <c r="F13" s="154"/>
       <c r="G13" s="109"/>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.4">
@@ -14492,10 +15403,10 @@
     </row>
     <row r="15" spans="2:10" ht="100.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D15" s="86"/>
-      <c r="E15" s="147" t="s">
+      <c r="E15" s="150" t="s">
         <v>333</v>
       </c>
-      <c r="F15" s="147"/>
+      <c r="F15" s="150"/>
       <c r="G15" s="108" t="s">
         <v>336</v>
       </c>
@@ -14510,21 +15421,21 @@
       <c r="F16" s="114"/>
       <c r="G16" s="114"/>
       <c r="H16" s="114"/>
-      <c r="I16" s="147" t="s">
+      <c r="I16" s="150" t="s">
         <v>345</v>
       </c>
-      <c r="J16" s="147"/>
+      <c r="J16" s="150"/>
     </row>
     <row r="17" spans="4:10" x14ac:dyDescent="0.4">
       <c r="D17" s="86"/>
       <c r="E17" s="120"/>
     </row>
     <row r="18" spans="4:10" ht="79.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E18" s="147" t="s">
+      <c r="E18" s="150" t="s">
         <v>164</v>
       </c>
-      <c r="F18" s="147"/>
-      <c r="G18" s="152" t="s">
+      <c r="F18" s="150"/>
+      <c r="G18" s="155" t="s">
         <v>163</v>
       </c>
       <c r="H18" s="93" t="s">
@@ -14533,28 +15444,28 @@
       <c r="I18" s="85" t="s">
         <v>165</v>
       </c>
-      <c r="J18" s="147" t="s">
+      <c r="J18" s="150" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="19" spans="4:10" ht="70.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E19" s="147"/>
-      <c r="F19" s="147"/>
-      <c r="G19" s="152"/>
-      <c r="H19" s="148" t="s">
+      <c r="E19" s="150"/>
+      <c r="F19" s="150"/>
+      <c r="G19" s="155"/>
+      <c r="H19" s="151" t="s">
         <v>167</v>
       </c>
-      <c r="I19" s="149"/>
-      <c r="J19" s="151"/>
+      <c r="I19" s="152"/>
+      <c r="J19" s="154"/>
     </row>
     <row r="20" spans="4:10" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="F20" s="92"/>
     </row>
     <row r="21" spans="4:10" s="81" customFormat="1" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E21" s="148" t="s">
+      <c r="E21" s="151" t="s">
         <v>149</v>
       </c>
-      <c r="F21" s="149"/>
+      <c r="F21" s="152"/>
       <c r="G21" s="83" t="s">
         <v>155</v>
       </c>
@@ -14565,10 +15476,10 @@
       </c>
     </row>
     <row r="23" spans="4:10" ht="100.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E23" s="148" t="s">
+      <c r="E23" s="151" t="s">
         <v>152</v>
       </c>
-      <c r="F23" s="149"/>
+      <c r="F23" s="152"/>
       <c r="G23" s="85" t="s">
         <v>156</v>
       </c>
@@ -14579,10 +15490,10 @@
       </c>
     </row>
     <row r="25" spans="4:10" ht="100.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E25" s="148" t="s">
+      <c r="E25" s="151" t="s">
         <v>154</v>
       </c>
-      <c r="F25" s="149"/>
+      <c r="F25" s="152"/>
       <c r="G25" s="84" t="s">
         <v>157</v>
       </c>
@@ -14642,10 +15553,10 @@
       </c>
     </row>
     <row r="3" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B3" s="156" t="s">
+      <c r="B3" s="159" t="s">
         <v>520</v>
       </c>
-      <c r="C3" s="153" t="s">
+      <c r="C3" s="156" t="s">
         <v>528</v>
       </c>
       <c r="D3" s="112" t="s">
@@ -14662,12 +15573,12 @@
       </c>
     </row>
     <row r="4" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B4" s="157"/>
-      <c r="C4" s="154"/>
-      <c r="D4" s="164" t="s">
+      <c r="B4" s="160"/>
+      <c r="C4" s="157"/>
+      <c r="D4" s="167" t="s">
         <v>445</v>
       </c>
-      <c r="E4" s="153" t="s">
+      <c r="E4" s="156" t="s">
         <v>529</v>
       </c>
       <c r="F4" s="68" t="s">
@@ -14678,10 +15589,10 @@
       </c>
     </row>
     <row r="5" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B5" s="157"/>
-      <c r="C5" s="154"/>
-      <c r="D5" s="169"/>
-      <c r="E5" s="154"/>
+      <c r="B5" s="160"/>
+      <c r="C5" s="157"/>
+      <c r="D5" s="172"/>
+      <c r="E5" s="157"/>
       <c r="F5" s="125" t="s">
         <v>532</v>
       </c>
@@ -14690,10 +15601,10 @@
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B6" s="157"/>
-      <c r="C6" s="154"/>
-      <c r="D6" s="169"/>
-      <c r="E6" s="154"/>
+      <c r="B6" s="160"/>
+      <c r="C6" s="157"/>
+      <c r="D6" s="172"/>
+      <c r="E6" s="157"/>
       <c r="F6" s="125" t="s">
         <v>534</v>
       </c>
@@ -14702,10 +15613,10 @@
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B7" s="157"/>
-      <c r="C7" s="154"/>
-      <c r="D7" s="165"/>
-      <c r="E7" s="155"/>
+      <c r="B7" s="160"/>
+      <c r="C7" s="157"/>
+      <c r="D7" s="168"/>
+      <c r="E7" s="158"/>
       <c r="F7" s="68" t="s">
         <v>536</v>
       </c>
@@ -14714,8 +15625,8 @@
       </c>
     </row>
     <row r="8" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B8" s="158"/>
-      <c r="C8" s="155"/>
+      <c r="B8" s="161"/>
+      <c r="C8" s="158"/>
       <c r="D8" s="95" t="s">
         <v>446</v>
       </c>
@@ -14733,40 +15644,40 @@
       <c r="B9" s="139" t="s">
         <v>523</v>
       </c>
-      <c r="C9" s="166" t="s">
+      <c r="C9" s="169" t="s">
         <v>524</v>
       </c>
-      <c r="D9" s="167"/>
-      <c r="E9" s="167"/>
-      <c r="F9" s="167"/>
-      <c r="G9" s="168"/>
+      <c r="D9" s="170"/>
+      <c r="E9" s="170"/>
+      <c r="F9" s="170"/>
+      <c r="G9" s="171"/>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B10" s="139" t="s">
         <v>521</v>
       </c>
-      <c r="C10" s="166" t="s">
+      <c r="C10" s="169" t="s">
         <v>522</v>
       </c>
-      <c r="D10" s="167"/>
-      <c r="E10" s="167"/>
-      <c r="F10" s="167"/>
-      <c r="G10" s="168"/>
+      <c r="D10" s="170"/>
+      <c r="E10" s="170"/>
+      <c r="F10" s="170"/>
+      <c r="G10" s="171"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B11" s="159"/>
-      <c r="C11" s="159"/>
-      <c r="D11" s="159"/>
-      <c r="E11" s="159"/>
-      <c r="F11" s="159"/>
-      <c r="G11" s="159"/>
+      <c r="B11" s="162"/>
+      <c r="C11" s="162"/>
+      <c r="D11" s="162"/>
+      <c r="E11" s="162"/>
+      <c r="F11" s="162"/>
+      <c r="G11" s="162"/>
       <c r="H11" s="117"/>
     </row>
     <row r="12" spans="2:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="156" t="s">
+      <c r="B12" s="159" t="s">
         <v>492</v>
       </c>
-      <c r="C12" s="153" t="s">
+      <c r="C12" s="156" t="s">
         <v>437</v>
       </c>
       <c r="D12" s="112" t="s">
@@ -14783,12 +15694,12 @@
       </c>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B13" s="157"/>
-      <c r="C13" s="154"/>
-      <c r="D13" s="164" t="s">
+      <c r="B13" s="160"/>
+      <c r="C13" s="157"/>
+      <c r="D13" s="167" t="s">
         <v>445</v>
       </c>
-      <c r="E13" s="153" t="s">
+      <c r="E13" s="156" t="s">
         <v>500</v>
       </c>
       <c r="F13" s="125" t="s">
@@ -14799,10 +15710,10 @@
       </c>
     </row>
     <row r="14" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B14" s="157"/>
-      <c r="C14" s="154"/>
-      <c r="D14" s="169"/>
-      <c r="E14" s="154"/>
+      <c r="B14" s="160"/>
+      <c r="C14" s="157"/>
+      <c r="D14" s="172"/>
+      <c r="E14" s="157"/>
       <c r="F14" s="68" t="s">
         <v>503</v>
       </c>
@@ -14811,10 +15722,10 @@
       </c>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B15" s="157"/>
-      <c r="C15" s="154"/>
-      <c r="D15" s="165"/>
-      <c r="E15" s="155"/>
+      <c r="B15" s="160"/>
+      <c r="C15" s="157"/>
+      <c r="D15" s="168"/>
+      <c r="E15" s="158"/>
       <c r="F15" s="68" t="s">
         <v>505</v>
       </c>
@@ -14823,12 +15734,12 @@
       </c>
     </row>
     <row r="16" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B16" s="157"/>
-      <c r="C16" s="154"/>
-      <c r="D16" s="164" t="s">
+      <c r="B16" s="160"/>
+      <c r="C16" s="157"/>
+      <c r="D16" s="167" t="s">
         <v>446</v>
       </c>
-      <c r="E16" s="164" t="s">
+      <c r="E16" s="167" t="s">
         <v>507</v>
       </c>
       <c r="F16" s="68" t="s">
@@ -14839,10 +15750,10 @@
       </c>
     </row>
     <row r="17" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B17" s="157"/>
-      <c r="C17" s="154"/>
-      <c r="D17" s="169"/>
-      <c r="E17" s="169"/>
+      <c r="B17" s="160"/>
+      <c r="C17" s="157"/>
+      <c r="D17" s="172"/>
+      <c r="E17" s="172"/>
       <c r="F17" s="68" t="s">
         <v>510</v>
       </c>
@@ -14851,10 +15762,10 @@
       </c>
     </row>
     <row r="18" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B18" s="157"/>
-      <c r="C18" s="154"/>
-      <c r="D18" s="169"/>
-      <c r="E18" s="169"/>
+      <c r="B18" s="160"/>
+      <c r="C18" s="157"/>
+      <c r="D18" s="172"/>
+      <c r="E18" s="172"/>
       <c r="F18" s="68" t="s">
         <v>512</v>
       </c>
@@ -14863,10 +15774,10 @@
       </c>
     </row>
     <row r="19" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B19" s="157"/>
-      <c r="C19" s="154"/>
-      <c r="D19" s="169"/>
-      <c r="E19" s="169"/>
+      <c r="B19" s="160"/>
+      <c r="C19" s="157"/>
+      <c r="D19" s="172"/>
+      <c r="E19" s="172"/>
       <c r="F19" s="68" t="s">
         <v>514</v>
       </c>
@@ -14875,10 +15786,10 @@
       </c>
     </row>
     <row r="20" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B20" s="157"/>
-      <c r="C20" s="154"/>
-      <c r="D20" s="169"/>
-      <c r="E20" s="169"/>
+      <c r="B20" s="160"/>
+      <c r="C20" s="157"/>
+      <c r="D20" s="172"/>
+      <c r="E20" s="172"/>
       <c r="F20" s="68" t="s">
         <v>516</v>
       </c>
@@ -14887,10 +15798,10 @@
       </c>
     </row>
     <row r="21" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B21" s="157"/>
-      <c r="C21" s="155"/>
-      <c r="D21" s="165"/>
-      <c r="E21" s="165"/>
+      <c r="B21" s="160"/>
+      <c r="C21" s="158"/>
+      <c r="D21" s="168"/>
+      <c r="E21" s="168"/>
       <c r="F21" s="68" t="s">
         <v>518</v>
       </c>
@@ -14899,16 +15810,16 @@
       </c>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B22" s="157"/>
-      <c r="C22" s="161"/>
-      <c r="D22" s="162"/>
-      <c r="E22" s="162"/>
-      <c r="F22" s="162"/>
-      <c r="G22" s="163"/>
+      <c r="B22" s="160"/>
+      <c r="C22" s="164"/>
+      <c r="D22" s="165"/>
+      <c r="E22" s="165"/>
+      <c r="F22" s="165"/>
+      <c r="G22" s="166"/>
     </row>
     <row r="23" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B23" s="157"/>
-      <c r="C23" s="153" t="s">
+      <c r="B23" s="160"/>
+      <c r="C23" s="156" t="s">
         <v>438</v>
       </c>
       <c r="D23" s="111" t="s">
@@ -14923,8 +15834,8 @@
       </c>
     </row>
     <row r="24" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B24" s="157"/>
-      <c r="C24" s="154"/>
+      <c r="B24" s="160"/>
+      <c r="C24" s="157"/>
       <c r="D24" s="111" t="s">
         <v>445</v>
       </c>
@@ -14937,8 +15848,8 @@
       </c>
     </row>
     <row r="25" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B25" s="158"/>
-      <c r="C25" s="155"/>
+      <c r="B25" s="161"/>
+      <c r="C25" s="158"/>
       <c r="D25" s="111" t="s">
         <v>446</v>
       </c>
@@ -14951,19 +15862,19 @@
       </c>
     </row>
     <row r="26" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B26" s="159"/>
-      <c r="C26" s="159"/>
-      <c r="D26" s="159"/>
-      <c r="E26" s="159"/>
-      <c r="F26" s="159"/>
-      <c r="G26" s="159"/>
+      <c r="B26" s="162"/>
+      <c r="C26" s="162"/>
+      <c r="D26" s="162"/>
+      <c r="E26" s="162"/>
+      <c r="F26" s="162"/>
+      <c r="G26" s="162"/>
       <c r="H26" s="117"/>
     </row>
     <row r="27" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B27" s="160" t="s">
+      <c r="B27" s="163" t="s">
         <v>466</v>
       </c>
-      <c r="C27" s="153" t="s">
+      <c r="C27" s="156" t="s">
         <v>436</v>
       </c>
       <c r="D27" s="112" t="s">
@@ -14980,8 +15891,8 @@
       </c>
     </row>
     <row r="28" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B28" s="160"/>
-      <c r="C28" s="154"/>
+      <c r="B28" s="163"/>
+      <c r="C28" s="157"/>
       <c r="D28" s="112" t="s">
         <v>445</v>
       </c>
@@ -14996,12 +15907,12 @@
       </c>
     </row>
     <row r="29" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B29" s="160"/>
-      <c r="C29" s="154"/>
-      <c r="D29" s="164" t="s">
+      <c r="B29" s="163"/>
+      <c r="C29" s="157"/>
+      <c r="D29" s="167" t="s">
         <v>446</v>
       </c>
-      <c r="E29" s="153" t="s">
+      <c r="E29" s="156" t="s">
         <v>480</v>
       </c>
       <c r="F29" s="67" t="s">
@@ -15012,10 +15923,10 @@
       </c>
     </row>
     <row r="30" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B30" s="160"/>
-      <c r="C30" s="154"/>
-      <c r="D30" s="165"/>
-      <c r="E30" s="155"/>
+      <c r="B30" s="163"/>
+      <c r="C30" s="157"/>
+      <c r="D30" s="168"/>
+      <c r="E30" s="158"/>
       <c r="F30" s="67" t="s">
         <v>483</v>
       </c>
@@ -15024,8 +15935,8 @@
       </c>
     </row>
     <row r="31" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B31" s="160"/>
-      <c r="C31" s="154"/>
+      <c r="B31" s="163"/>
+      <c r="C31" s="157"/>
       <c r="D31" s="112" t="s">
         <v>458</v>
       </c>
@@ -15040,8 +15951,8 @@
       </c>
     </row>
     <row r="32" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B32" s="160"/>
-      <c r="C32" s="155"/>
+      <c r="B32" s="163"/>
+      <c r="C32" s="158"/>
       <c r="D32" s="112" t="s">
         <v>459</v>
       </c>
@@ -15056,7 +15967,7 @@
       </c>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B33" s="160"/>
+      <c r="B33" s="163"/>
       <c r="C33" s="130"/>
       <c r="D33" s="127"/>
       <c r="E33" s="130"/>
@@ -15064,8 +15975,8 @@
       <c r="G33" s="130"/>
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B34" s="160"/>
-      <c r="C34" s="153" t="s">
+      <c r="B34" s="163"/>
+      <c r="C34" s="156" t="s">
         <v>144</v>
       </c>
       <c r="D34" s="95" t="s">
@@ -15080,8 +15991,8 @@
       </c>
     </row>
     <row r="35" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B35" s="156"/>
-      <c r="C35" s="154"/>
+      <c r="B35" s="159"/>
+      <c r="C35" s="157"/>
       <c r="D35" s="111" t="s">
         <v>445</v>
       </c>
@@ -15094,19 +16005,19 @@
       </c>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B36" s="159"/>
-      <c r="C36" s="159"/>
-      <c r="D36" s="159"/>
-      <c r="E36" s="159"/>
-      <c r="F36" s="159"/>
-      <c r="G36" s="159"/>
-      <c r="H36" s="159"/>
+      <c r="B36" s="162"/>
+      <c r="C36" s="162"/>
+      <c r="D36" s="162"/>
+      <c r="E36" s="162"/>
+      <c r="F36" s="162"/>
+      <c r="G36" s="162"/>
+      <c r="H36" s="162"/>
     </row>
     <row r="37" spans="2:8" ht="93.6" x14ac:dyDescent="0.3">
-      <c r="B37" s="160" t="s">
+      <c r="B37" s="163" t="s">
         <v>465</v>
       </c>
-      <c r="C37" s="153" t="s">
+      <c r="C37" s="156" t="s">
         <v>435</v>
       </c>
       <c r="D37" s="95" t="s">
@@ -15121,13 +16032,13 @@
       <c r="G37" s="113" t="s">
         <v>462</v>
       </c>
-      <c r="H37" s="170" t="s">
+      <c r="H37" s="173" t="s">
         <v>475</v>
       </c>
     </row>
     <row r="38" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B38" s="160"/>
-      <c r="C38" s="155"/>
+      <c r="B38" s="163"/>
+      <c r="C38" s="158"/>
       <c r="D38" s="95" t="s">
         <v>445</v>
       </c>
@@ -15138,19 +16049,19 @@
       <c r="G38" s="138" t="s">
         <v>464</v>
       </c>
-      <c r="H38" s="171"/>
+      <c r="H38" s="174"/>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B39" s="160"/>
-      <c r="C39" s="161"/>
-      <c r="D39" s="162"/>
-      <c r="E39" s="162"/>
-      <c r="F39" s="162"/>
-      <c r="G39" s="163"/>
+      <c r="B39" s="163"/>
+      <c r="C39" s="164"/>
+      <c r="D39" s="165"/>
+      <c r="E39" s="165"/>
+      <c r="F39" s="165"/>
+      <c r="G39" s="166"/>
     </row>
     <row r="40" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B40" s="160"/>
-      <c r="C40" s="153" t="s">
+      <c r="B40" s="163"/>
+      <c r="C40" s="156" t="s">
         <v>434</v>
       </c>
       <c r="D40" s="95" t="s">
@@ -15165,8 +16076,8 @@
       </c>
     </row>
     <row r="41" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B41" s="160"/>
-      <c r="C41" s="154"/>
+      <c r="B41" s="163"/>
+      <c r="C41" s="157"/>
       <c r="D41" s="95" t="s">
         <v>445</v>
       </c>
@@ -15179,8 +16090,8 @@
       </c>
     </row>
     <row r="42" spans="2:8" ht="93.6" x14ac:dyDescent="0.3">
-      <c r="B42" s="160"/>
-      <c r="C42" s="154"/>
+      <c r="B42" s="163"/>
+      <c r="C42" s="157"/>
       <c r="D42" s="95" t="s">
         <v>446</v>
       </c>
@@ -15195,8 +16106,8 @@
       </c>
     </row>
     <row r="43" spans="2:8" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="B43" s="160"/>
-      <c r="C43" s="154"/>
+      <c r="B43" s="163"/>
+      <c r="C43" s="157"/>
       <c r="D43" s="95" t="s">
         <v>458</v>
       </c>
@@ -15211,8 +16122,8 @@
       </c>
     </row>
     <row r="44" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B44" s="160"/>
-      <c r="C44" s="155"/>
+      <c r="B44" s="163"/>
+      <c r="C44" s="158"/>
       <c r="D44" s="95" t="s">
         <v>459</v>
       </c>
@@ -15227,19 +16138,19 @@
       </c>
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B45" s="159"/>
-      <c r="C45" s="159"/>
-      <c r="D45" s="159"/>
-      <c r="E45" s="159"/>
-      <c r="F45" s="159"/>
-      <c r="G45" s="159"/>
+      <c r="B45" s="162"/>
+      <c r="C45" s="162"/>
+      <c r="D45" s="162"/>
+      <c r="E45" s="162"/>
+      <c r="F45" s="162"/>
+      <c r="G45" s="162"/>
       <c r="H45" s="117"/>
     </row>
     <row r="46" spans="2:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="156" t="s">
+      <c r="B46" s="159" t="s">
         <v>541</v>
       </c>
-      <c r="C46" s="153" t="s">
+      <c r="C46" s="156" t="s">
         <v>440</v>
       </c>
       <c r="D46" s="95" t="s">
@@ -15256,8 +16167,8 @@
       </c>
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B47" s="157"/>
-      <c r="C47" s="154"/>
+      <c r="B47" s="160"/>
+      <c r="C47" s="157"/>
       <c r="D47" s="95" t="s">
         <v>445</v>
       </c>
@@ -15272,8 +16183,8 @@
       </c>
     </row>
     <row r="48" spans="2:8" ht="78" x14ac:dyDescent="0.3">
-      <c r="B48" s="157"/>
-      <c r="C48" s="154"/>
+      <c r="B48" s="160"/>
+      <c r="C48" s="157"/>
       <c r="D48" s="95" t="s">
         <v>446</v>
       </c>
@@ -15288,8 +16199,8 @@
       </c>
     </row>
     <row r="49" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B49" s="157"/>
-      <c r="C49" s="154"/>
+      <c r="B49" s="160"/>
+      <c r="C49" s="157"/>
       <c r="D49" s="95" t="s">
         <v>458</v>
       </c>
@@ -15304,8 +16215,8 @@
       </c>
     </row>
     <row r="50" spans="2:7" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B50" s="157"/>
-      <c r="C50" s="154"/>
+      <c r="B50" s="160"/>
+      <c r="C50" s="157"/>
       <c r="D50" s="95" t="s">
         <v>459</v>
       </c>
@@ -15320,8 +16231,8 @@
       </c>
     </row>
     <row r="51" spans="2:7" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="B51" s="157"/>
-      <c r="C51" s="154"/>
+      <c r="B51" s="160"/>
+      <c r="C51" s="157"/>
       <c r="D51" s="95" t="s">
         <v>553</v>
       </c>
@@ -15336,8 +16247,8 @@
       </c>
     </row>
     <row r="52" spans="2:7" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="B52" s="157"/>
-      <c r="C52" s="154"/>
+      <c r="B52" s="160"/>
+      <c r="C52" s="157"/>
       <c r="D52" s="95" t="s">
         <v>554</v>
       </c>
@@ -15352,8 +16263,8 @@
       </c>
     </row>
     <row r="53" spans="2:7" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B53" s="158"/>
-      <c r="C53" s="155"/>
+      <c r="B53" s="161"/>
+      <c r="C53" s="158"/>
       <c r="D53" s="95" t="s">
         <v>565</v>
       </c>
@@ -15419,10 +16330,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.4">
-      <c r="B2" s="150" t="s">
+      <c r="B2" s="153" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="150"/>
+      <c r="C2" s="153"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C3" s="7" t="s">
@@ -15430,10 +16341,10 @@
       </c>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.4">
-      <c r="B4" s="150" t="s">
+      <c r="B4" s="153" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="150"/>
+      <c r="C4" s="153"/>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C5" s="7" t="s">
@@ -15441,10 +16352,10 @@
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.4">
-      <c r="B6" s="150" t="s">
+      <c r="B6" s="153" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="150"/>
+      <c r="C6" s="153"/>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C7" s="7" t="s">
@@ -15452,10 +16363,10 @@
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.4">
-      <c r="B8" s="150" t="s">
+      <c r="B8" s="153" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="150"/>
+      <c r="C8" s="153"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C9" s="7" t="s">
@@ -15463,10 +16374,10 @@
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.4">
-      <c r="B10" s="150" t="s">
+      <c r="B10" s="153" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="150"/>
+      <c r="C10" s="153"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.4">
       <c r="D11" s="80" t="s">
@@ -15488,10 +16399,10 @@
       <c r="F13" s="119" t="s">
         <v>339</v>
       </c>
-      <c r="G13" s="172" t="s">
+      <c r="G13" s="175" t="s">
         <v>340</v>
       </c>
-      <c r="H13" s="173"/>
+      <c r="H13" s="176"/>
     </row>
     <row r="14" spans="2:8" ht="150" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D14" s="86"/>
@@ -15499,10 +16410,10 @@
       <c r="F14" s="87" t="s">
         <v>341</v>
       </c>
-      <c r="G14" s="148" t="s">
+      <c r="G14" s="151" t="s">
         <v>342</v>
       </c>
-      <c r="H14" s="174"/>
+      <c r="H14" s="177"/>
     </row>
     <row r="15" spans="2:8" ht="150" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D15" s="86"/>
@@ -15510,10 +16421,10 @@
       <c r="F15" s="87" t="s">
         <v>343</v>
       </c>
-      <c r="G15" s="148" t="s">
+      <c r="G15" s="151" t="s">
         <v>344</v>
       </c>
-      <c r="H15" s="174"/>
+      <c r="H15" s="177"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.4">
       <c r="D16" s="86"/>
@@ -15526,8 +16437,8 @@
       <c r="D17" s="86"/>
       <c r="E17" s="86"/>
       <c r="F17" s="87"/>
-      <c r="G17" s="151"/>
-      <c r="H17" s="151"/>
+      <c r="G17" s="154"/>
+      <c r="H17" s="154"/>
     </row>
     <row r="18" spans="4:8" x14ac:dyDescent="0.4">
       <c r="D18" s="86"/>
@@ -15541,10 +16452,10 @@
       <c r="F19" s="87" t="s">
         <v>158</v>
       </c>
-      <c r="G19" s="147" t="s">
+      <c r="G19" s="150" t="s">
         <v>159</v>
       </c>
-      <c r="H19" s="151"/>
+      <c r="H19" s="154"/>
     </row>
     <row r="20" spans="4:8" x14ac:dyDescent="0.4">
       <c r="H20" s="7"/>
@@ -15553,10 +16464,10 @@
       <c r="F21" s="89" t="s">
         <v>160</v>
       </c>
-      <c r="G21" s="148" t="s">
+      <c r="G21" s="151" t="s">
         <v>161</v>
       </c>
-      <c r="H21" s="149"/>
+      <c r="H21" s="152"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -15625,14 +16536,14 @@
       </c>
     </row>
     <row r="3" spans="2:11" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="176">
+      <c r="B3" s="179">
         <v>1</v>
       </c>
-      <c r="C3" s="176"/>
-      <c r="D3" s="164" t="s">
+      <c r="C3" s="179"/>
+      <c r="D3" s="167" t="s">
         <v>444</v>
       </c>
-      <c r="E3" s="164" t="s">
+      <c r="E3" s="167" t="s">
         <v>575</v>
       </c>
       <c r="F3" s="68" t="s">
@@ -15642,21 +16553,21 @@
         <v>576</v>
       </c>
       <c r="H3" s="140"/>
-      <c r="I3" s="175" t="s">
+      <c r="I3" s="178" t="s">
         <v>636</v>
       </c>
-      <c r="J3" s="179" t="s">
+      <c r="J3" s="182" t="s">
         <v>640</v>
       </c>
-      <c r="K3" s="179" t="s">
+      <c r="K3" s="182" t="s">
         <v>641</v>
       </c>
     </row>
     <row r="4" spans="2:11" ht="78" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="177"/>
-      <c r="C4" s="177"/>
-      <c r="D4" s="169"/>
-      <c r="E4" s="169"/>
+      <c r="B4" s="180"/>
+      <c r="C4" s="180"/>
+      <c r="D4" s="172"/>
+      <c r="E4" s="172"/>
       <c r="F4" s="68" t="s">
         <v>577</v>
       </c>
@@ -15664,15 +16575,15 @@
         <v>578</v>
       </c>
       <c r="H4" s="140"/>
-      <c r="I4" s="175"/>
-      <c r="J4" s="179"/>
-      <c r="K4" s="179"/>
+      <c r="I4" s="178"/>
+      <c r="J4" s="182"/>
+      <c r="K4" s="182"/>
     </row>
     <row r="5" spans="2:11" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B5" s="177"/>
-      <c r="C5" s="177"/>
-      <c r="D5" s="165"/>
-      <c r="E5" s="165"/>
+      <c r="B5" s="180"/>
+      <c r="C5" s="180"/>
+      <c r="D5" s="168"/>
+      <c r="E5" s="168"/>
       <c r="F5" s="68" t="s">
         <v>579</v>
       </c>
@@ -15680,17 +16591,17 @@
         <v>580</v>
       </c>
       <c r="H5" s="140"/>
-      <c r="I5" s="175"/>
-      <c r="J5" s="179"/>
-      <c r="K5" s="179"/>
+      <c r="I5" s="178"/>
+      <c r="J5" s="182"/>
+      <c r="K5" s="182"/>
     </row>
     <row r="6" spans="2:11" ht="171.6" x14ac:dyDescent="0.3">
-      <c r="B6" s="177"/>
-      <c r="C6" s="177"/>
-      <c r="D6" s="164" t="s">
+      <c r="B6" s="180"/>
+      <c r="C6" s="180"/>
+      <c r="D6" s="167" t="s">
         <v>445</v>
       </c>
-      <c r="E6" s="164" t="s">
+      <c r="E6" s="167" t="s">
         <v>581</v>
       </c>
       <c r="F6" s="68" t="s">
@@ -15700,15 +16611,15 @@
         <v>583</v>
       </c>
       <c r="H6" s="140"/>
-      <c r="I6" s="175"/>
-      <c r="J6" s="179"/>
-      <c r="K6" s="179"/>
+      <c r="I6" s="178"/>
+      <c r="J6" s="182"/>
+      <c r="K6" s="182"/>
     </row>
     <row r="7" spans="2:11" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B7" s="177"/>
-      <c r="C7" s="177"/>
-      <c r="D7" s="165"/>
-      <c r="E7" s="165"/>
+      <c r="B7" s="180"/>
+      <c r="C7" s="180"/>
+      <c r="D7" s="168"/>
+      <c r="E7" s="168"/>
       <c r="F7" s="13" t="s">
         <v>584</v>
       </c>
@@ -15716,13 +16627,13 @@
         <v>585</v>
       </c>
       <c r="H7" s="83"/>
-      <c r="I7" s="175"/>
-      <c r="J7" s="179"/>
-      <c r="K7" s="179"/>
+      <c r="I7" s="178"/>
+      <c r="J7" s="182"/>
+      <c r="K7" s="182"/>
     </row>
     <row r="8" spans="2:11" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B8" s="177"/>
-      <c r="C8" s="177"/>
+      <c r="B8" s="180"/>
+      <c r="C8" s="180"/>
       <c r="D8" s="95" t="s">
         <v>446</v>
       </c>
@@ -15736,17 +16647,17 @@
         <v>588</v>
       </c>
       <c r="H8" s="83"/>
-      <c r="I8" s="175"/>
-      <c r="J8" s="179"/>
-      <c r="K8" s="179"/>
+      <c r="I8" s="178"/>
+      <c r="J8" s="182"/>
+      <c r="K8" s="182"/>
     </row>
     <row r="9" spans="2:11" ht="78" x14ac:dyDescent="0.3">
-      <c r="B9" s="177"/>
-      <c r="C9" s="177"/>
-      <c r="D9" s="164" t="s">
+      <c r="B9" s="180"/>
+      <c r="C9" s="180"/>
+      <c r="D9" s="167" t="s">
         <v>458</v>
       </c>
-      <c r="E9" s="164" t="s">
+      <c r="E9" s="167" t="s">
         <v>589</v>
       </c>
       <c r="F9" s="13" t="s">
@@ -15756,15 +16667,15 @@
         <v>643</v>
       </c>
       <c r="H9" s="83"/>
-      <c r="I9" s="175"/>
-      <c r="J9" s="179"/>
-      <c r="K9" s="179"/>
+      <c r="I9" s="178"/>
+      <c r="J9" s="182"/>
+      <c r="K9" s="182"/>
     </row>
     <row r="10" spans="2:11" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="B10" s="177"/>
-      <c r="C10" s="177"/>
-      <c r="D10" s="165"/>
-      <c r="E10" s="165"/>
+      <c r="B10" s="180"/>
+      <c r="C10" s="180"/>
+      <c r="D10" s="168"/>
+      <c r="E10" s="168"/>
       <c r="F10" s="13" t="s">
         <v>546</v>
       </c>
@@ -15772,17 +16683,17 @@
         <v>595</v>
       </c>
       <c r="H10" s="83"/>
-      <c r="I10" s="175"/>
-      <c r="J10" s="179"/>
-      <c r="K10" s="179"/>
+      <c r="I10" s="178"/>
+      <c r="J10" s="182"/>
+      <c r="K10" s="182"/>
     </row>
     <row r="11" spans="2:11" ht="93.6" x14ac:dyDescent="0.3">
-      <c r="B11" s="177"/>
-      <c r="C11" s="177"/>
-      <c r="D11" s="164" t="s">
+      <c r="B11" s="180"/>
+      <c r="C11" s="180"/>
+      <c r="D11" s="167" t="s">
         <v>459</v>
       </c>
-      <c r="E11" s="164" t="s">
+      <c r="E11" s="167" t="s">
         <v>591</v>
       </c>
       <c r="F11" s="13" t="s">
@@ -15792,15 +16703,15 @@
         <v>644</v>
       </c>
       <c r="H11" s="83"/>
-      <c r="I11" s="175"/>
-      <c r="J11" s="179"/>
-      <c r="K11" s="179"/>
+      <c r="I11" s="178"/>
+      <c r="J11" s="182"/>
+      <c r="K11" s="182"/>
     </row>
     <row r="12" spans="2:11" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="B12" s="177"/>
-      <c r="C12" s="177"/>
-      <c r="D12" s="169"/>
-      <c r="E12" s="169"/>
+      <c r="B12" s="180"/>
+      <c r="C12" s="180"/>
+      <c r="D12" s="172"/>
+      <c r="E12" s="172"/>
       <c r="F12" s="13" t="s">
         <v>551</v>
       </c>
@@ -15808,15 +16719,15 @@
         <v>593</v>
       </c>
       <c r="H12" s="83"/>
-      <c r="I12" s="175"/>
-      <c r="J12" s="179"/>
-      <c r="K12" s="179"/>
+      <c r="I12" s="178"/>
+      <c r="J12" s="182"/>
+      <c r="K12" s="182"/>
     </row>
     <row r="13" spans="2:11" ht="140.4" x14ac:dyDescent="0.3">
-      <c r="B13" s="177"/>
-      <c r="C13" s="177"/>
-      <c r="D13" s="165"/>
-      <c r="E13" s="165"/>
+      <c r="B13" s="180"/>
+      <c r="C13" s="180"/>
+      <c r="D13" s="168"/>
+      <c r="E13" s="168"/>
       <c r="F13" s="13" t="s">
         <v>594</v>
       </c>
@@ -15826,17 +16737,17 @@
       <c r="H13" s="83" t="s">
         <v>599</v>
       </c>
-      <c r="I13" s="175"/>
-      <c r="J13" s="179"/>
-      <c r="K13" s="179"/>
+      <c r="I13" s="178"/>
+      <c r="J13" s="182"/>
+      <c r="K13" s="182"/>
     </row>
     <row r="14" spans="2:11" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="B14" s="177"/>
-      <c r="C14" s="177"/>
-      <c r="D14" s="164" t="s">
+      <c r="B14" s="180"/>
+      <c r="C14" s="180"/>
+      <c r="D14" s="167" t="s">
         <v>553</v>
       </c>
-      <c r="E14" s="164" t="s">
+      <c r="E14" s="167" t="s">
         <v>597</v>
       </c>
       <c r="F14" s="13" t="s">
@@ -15846,15 +16757,15 @@
         <v>600</v>
       </c>
       <c r="H14" s="83"/>
-      <c r="I14" s="175"/>
-      <c r="J14" s="179"/>
-      <c r="K14" s="179"/>
+      <c r="I14" s="178"/>
+      <c r="J14" s="182"/>
+      <c r="K14" s="182"/>
     </row>
     <row r="15" spans="2:11" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="B15" s="177"/>
-      <c r="C15" s="177"/>
-      <c r="D15" s="169"/>
-      <c r="E15" s="169"/>
+      <c r="B15" s="180"/>
+      <c r="C15" s="180"/>
+      <c r="D15" s="172"/>
+      <c r="E15" s="172"/>
       <c r="F15" s="13" t="s">
         <v>601</v>
       </c>
@@ -15862,15 +16773,15 @@
         <v>602</v>
       </c>
       <c r="H15" s="83"/>
-      <c r="I15" s="175"/>
-      <c r="J15" s="179"/>
-      <c r="K15" s="179"/>
+      <c r="I15" s="178"/>
+      <c r="J15" s="182"/>
+      <c r="K15" s="182"/>
     </row>
     <row r="16" spans="2:11" ht="140.4" x14ac:dyDescent="0.3">
-      <c r="B16" s="177"/>
-      <c r="C16" s="177"/>
-      <c r="D16" s="169"/>
-      <c r="E16" s="169"/>
+      <c r="B16" s="180"/>
+      <c r="C16" s="180"/>
+      <c r="D16" s="172"/>
+      <c r="E16" s="172"/>
       <c r="F16" s="13" t="s">
         <v>603</v>
       </c>
@@ -15878,15 +16789,15 @@
         <v>604</v>
       </c>
       <c r="H16" s="83"/>
-      <c r="I16" s="175"/>
-      <c r="J16" s="179"/>
-      <c r="K16" s="179"/>
+      <c r="I16" s="178"/>
+      <c r="J16" s="182"/>
+      <c r="K16" s="182"/>
     </row>
     <row r="17" spans="2:11" ht="78" x14ac:dyDescent="0.3">
-      <c r="B17" s="177"/>
-      <c r="C17" s="177"/>
-      <c r="D17" s="165"/>
-      <c r="E17" s="165"/>
+      <c r="B17" s="180"/>
+      <c r="C17" s="180"/>
+      <c r="D17" s="168"/>
+      <c r="E17" s="168"/>
       <c r="F17" s="13" t="s">
         <v>594</v>
       </c>
@@ -15894,13 +16805,13 @@
         <v>605</v>
       </c>
       <c r="H17" s="83"/>
-      <c r="I17" s="175"/>
-      <c r="J17" s="179"/>
-      <c r="K17" s="179"/>
+      <c r="I17" s="178"/>
+      <c r="J17" s="182"/>
+      <c r="K17" s="182"/>
     </row>
     <row r="18" spans="2:11" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="B18" s="177"/>
-      <c r="C18" s="177"/>
+      <c r="B18" s="180"/>
+      <c r="C18" s="180"/>
       <c r="D18" s="95" t="s">
         <v>554</v>
       </c>
@@ -15914,17 +16825,17 @@
         <v>610</v>
       </c>
       <c r="H18" s="83"/>
-      <c r="I18" s="175"/>
-      <c r="J18" s="179"/>
-      <c r="K18" s="179"/>
+      <c r="I18" s="178"/>
+      <c r="J18" s="182"/>
+      <c r="K18" s="182"/>
     </row>
     <row r="19" spans="2:11" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B19" s="177"/>
-      <c r="C19" s="177"/>
-      <c r="D19" s="164" t="s">
+      <c r="B19" s="180"/>
+      <c r="C19" s="180"/>
+      <c r="D19" s="167" t="s">
         <v>565</v>
       </c>
-      <c r="E19" s="164" t="s">
+      <c r="E19" s="167" t="s">
         <v>611</v>
       </c>
       <c r="F19" s="13" t="s">
@@ -15934,15 +16845,15 @@
         <v>612</v>
       </c>
       <c r="H19" s="83"/>
-      <c r="I19" s="175"/>
-      <c r="J19" s="179"/>
-      <c r="K19" s="179"/>
+      <c r="I19" s="178"/>
+      <c r="J19" s="182"/>
+      <c r="K19" s="182"/>
     </row>
     <row r="20" spans="2:11" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B20" s="177"/>
-      <c r="C20" s="177"/>
-      <c r="D20" s="169"/>
-      <c r="E20" s="169"/>
+      <c r="B20" s="180"/>
+      <c r="C20" s="180"/>
+      <c r="D20" s="172"/>
+      <c r="E20" s="172"/>
       <c r="F20" s="13" t="s">
         <v>613</v>
       </c>
@@ -15950,15 +16861,15 @@
         <v>614</v>
       </c>
       <c r="H20" s="83"/>
-      <c r="I20" s="175"/>
-      <c r="J20" s="179"/>
-      <c r="K20" s="179"/>
+      <c r="I20" s="178"/>
+      <c r="J20" s="182"/>
+      <c r="K20" s="182"/>
     </row>
     <row r="21" spans="2:11" ht="78" x14ac:dyDescent="0.3">
-      <c r="B21" s="177"/>
-      <c r="C21" s="177"/>
-      <c r="D21" s="169"/>
-      <c r="E21" s="169"/>
+      <c r="B21" s="180"/>
+      <c r="C21" s="180"/>
+      <c r="D21" s="172"/>
+      <c r="E21" s="172"/>
       <c r="F21" s="13" t="s">
         <v>615</v>
       </c>
@@ -15966,15 +16877,15 @@
         <v>616</v>
       </c>
       <c r="H21" s="83"/>
-      <c r="I21" s="175"/>
-      <c r="J21" s="179"/>
-      <c r="K21" s="179"/>
+      <c r="I21" s="178"/>
+      <c r="J21" s="182"/>
+      <c r="K21" s="182"/>
     </row>
     <row r="22" spans="2:11" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B22" s="177"/>
-      <c r="C22" s="177"/>
-      <c r="D22" s="169"/>
-      <c r="E22" s="169"/>
+      <c r="B22" s="180"/>
+      <c r="C22" s="180"/>
+      <c r="D22" s="172"/>
+      <c r="E22" s="172"/>
       <c r="F22" s="13" t="s">
         <v>617</v>
       </c>
@@ -15982,15 +16893,15 @@
         <v>618</v>
       </c>
       <c r="H22" s="83"/>
-      <c r="I22" s="175"/>
-      <c r="J22" s="179"/>
-      <c r="K22" s="179"/>
+      <c r="I22" s="178"/>
+      <c r="J22" s="182"/>
+      <c r="K22" s="182"/>
     </row>
     <row r="23" spans="2:11" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B23" s="177"/>
-      <c r="C23" s="177"/>
-      <c r="D23" s="165"/>
-      <c r="E23" s="165"/>
+      <c r="B23" s="180"/>
+      <c r="C23" s="180"/>
+      <c r="D23" s="168"/>
+      <c r="E23" s="168"/>
       <c r="F23" s="13" t="s">
         <v>619</v>
       </c>
@@ -15998,17 +16909,17 @@
         <v>620</v>
       </c>
       <c r="H23" s="83"/>
-      <c r="I23" s="175"/>
-      <c r="J23" s="179"/>
-      <c r="K23" s="179"/>
+      <c r="I23" s="178"/>
+      <c r="J23" s="182"/>
+      <c r="K23" s="182"/>
     </row>
     <row r="24" spans="2:11" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B24" s="177"/>
-      <c r="C24" s="177"/>
-      <c r="D24" s="164" t="s">
+      <c r="B24" s="180"/>
+      <c r="C24" s="180"/>
+      <c r="D24" s="167" t="s">
         <v>590</v>
       </c>
-      <c r="E24" s="164" t="s">
+      <c r="E24" s="167" t="s">
         <v>621</v>
       </c>
       <c r="F24" s="13" t="s">
@@ -16018,15 +16929,15 @@
         <v>623</v>
       </c>
       <c r="H24" s="83"/>
-      <c r="I24" s="175"/>
-      <c r="J24" s="179"/>
-      <c r="K24" s="179"/>
+      <c r="I24" s="178"/>
+      <c r="J24" s="182"/>
+      <c r="K24" s="182"/>
     </row>
     <row r="25" spans="2:11" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B25" s="177"/>
-      <c r="C25" s="177"/>
-      <c r="D25" s="169"/>
-      <c r="E25" s="169"/>
+      <c r="B25" s="180"/>
+      <c r="C25" s="180"/>
+      <c r="D25" s="172"/>
+      <c r="E25" s="172"/>
       <c r="F25" s="13" t="s">
         <v>624</v>
       </c>
@@ -16034,15 +16945,15 @@
         <v>625</v>
       </c>
       <c r="H25" s="83"/>
-      <c r="I25" s="175"/>
-      <c r="J25" s="179"/>
-      <c r="K25" s="179"/>
+      <c r="I25" s="178"/>
+      <c r="J25" s="182"/>
+      <c r="K25" s="182"/>
     </row>
     <row r="26" spans="2:11" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B26" s="177"/>
-      <c r="C26" s="177"/>
-      <c r="D26" s="165"/>
-      <c r="E26" s="165"/>
+      <c r="B26" s="180"/>
+      <c r="C26" s="180"/>
+      <c r="D26" s="168"/>
+      <c r="E26" s="168"/>
       <c r="F26" s="13" t="s">
         <v>594</v>
       </c>
@@ -16050,13 +16961,13 @@
         <v>626</v>
       </c>
       <c r="H26" s="83"/>
-      <c r="I26" s="175"/>
-      <c r="J26" s="179"/>
-      <c r="K26" s="179"/>
+      <c r="I26" s="178"/>
+      <c r="J26" s="182"/>
+      <c r="K26" s="182"/>
     </row>
     <row r="27" spans="2:11" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B27" s="177"/>
-      <c r="C27" s="177"/>
+      <c r="B27" s="180"/>
+      <c r="C27" s="180"/>
       <c r="D27" s="95" t="s">
         <v>606</v>
       </c>
@@ -16068,13 +16979,13 @@
         <v>629</v>
       </c>
       <c r="H27" s="83"/>
-      <c r="I27" s="175"/>
-      <c r="J27" s="179"/>
-      <c r="K27" s="179"/>
+      <c r="I27" s="178"/>
+      <c r="J27" s="182"/>
+      <c r="K27" s="182"/>
     </row>
     <row r="28" spans="2:11" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="B28" s="177"/>
-      <c r="C28" s="177"/>
+      <c r="B28" s="180"/>
+      <c r="C28" s="180"/>
       <c r="D28" s="95" t="s">
         <v>607</v>
       </c>
@@ -16088,13 +16999,13 @@
         <v>632</v>
       </c>
       <c r="H28" s="83"/>
-      <c r="I28" s="175"/>
-      <c r="J28" s="179"/>
-      <c r="K28" s="179"/>
+      <c r="I28" s="178"/>
+      <c r="J28" s="182"/>
+      <c r="K28" s="182"/>
     </row>
     <row r="29" spans="2:11" ht="78" x14ac:dyDescent="0.3">
-      <c r="B29" s="178"/>
-      <c r="C29" s="178"/>
+      <c r="B29" s="181"/>
+      <c r="C29" s="181"/>
       <c r="D29" s="95" t="s">
         <v>627</v>
       </c>
@@ -16108,12 +17019,18 @@
         <v>635</v>
       </c>
       <c r="H29" s="83"/>
-      <c r="I29" s="175"/>
-      <c r="J29" s="179"/>
-      <c r="K29" s="179"/>
+      <c r="I29" s="178"/>
+      <c r="J29" s="182"/>
+      <c r="K29" s="182"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="D11:D13"/>
+    <mergeCell ref="D3:D5"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="I3:I29"/>
+    <mergeCell ref="C3:C29"/>
     <mergeCell ref="B3:B29"/>
     <mergeCell ref="K3:K29"/>
     <mergeCell ref="J3:J29"/>
@@ -16127,12 +17044,6 @@
     <mergeCell ref="E6:E7"/>
     <mergeCell ref="E9:E10"/>
     <mergeCell ref="E11:E13"/>
-    <mergeCell ref="D11:D13"/>
-    <mergeCell ref="D3:D5"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="I3:I29"/>
-    <mergeCell ref="C3:C29"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -17436,10 +18347,10 @@
     </row>
     <row r="12" spans="2:118" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B12" s="17"/>
-      <c r="C12" s="186" t="s">
+      <c r="C12" s="189" t="s">
         <v>59</v>
       </c>
-      <c r="D12" s="186" t="s">
+      <c r="D12" s="189" t="s">
         <v>60</v>
       </c>
       <c r="E12" s="183" t="s">
@@ -17464,16 +18375,16 @@
       <c r="R12" s="184"/>
       <c r="S12" s="184"/>
       <c r="T12" s="184"/>
-      <c r="U12" s="189"/>
-      <c r="V12" s="180" t="s">
+      <c r="U12" s="192"/>
+      <c r="V12" s="186" t="s">
         <v>64</v>
       </c>
-      <c r="W12" s="181"/>
-      <c r="X12" s="181"/>
-      <c r="Y12" s="181"/>
-      <c r="Z12" s="181"/>
-      <c r="AA12" s="181"/>
-      <c r="AB12" s="182"/>
+      <c r="W12" s="187"/>
+      <c r="X12" s="187"/>
+      <c r="Y12" s="187"/>
+      <c r="Z12" s="187"/>
+      <c r="AA12" s="187"/>
+      <c r="AB12" s="188"/>
       <c r="AC12" s="183" t="s">
         <v>65</v>
       </c>
@@ -17482,106 +18393,106 @@
       <c r="AF12" s="184"/>
       <c r="AG12" s="184"/>
       <c r="AH12" s="184"/>
-      <c r="AI12" s="189"/>
-      <c r="AJ12" s="190" t="s">
+      <c r="AI12" s="192"/>
+      <c r="AJ12" s="193" t="s">
         <v>66</v>
       </c>
-      <c r="AK12" s="181"/>
-      <c r="AL12" s="181"/>
-      <c r="AM12" s="181"/>
-      <c r="AN12" s="181"/>
-      <c r="AO12" s="181"/>
-      <c r="AP12" s="182"/>
-      <c r="AQ12" s="180" t="s">
+      <c r="AK12" s="187"/>
+      <c r="AL12" s="187"/>
+      <c r="AM12" s="187"/>
+      <c r="AN12" s="187"/>
+      <c r="AO12" s="187"/>
+      <c r="AP12" s="188"/>
+      <c r="AQ12" s="186" t="s">
         <v>67</v>
       </c>
-      <c r="AR12" s="181"/>
-      <c r="AS12" s="181"/>
-      <c r="AT12" s="181"/>
-      <c r="AU12" s="181"/>
-      <c r="AV12" s="181"/>
-      <c r="AW12" s="182"/>
-      <c r="AX12" s="180" t="s">
+      <c r="AR12" s="187"/>
+      <c r="AS12" s="187"/>
+      <c r="AT12" s="187"/>
+      <c r="AU12" s="187"/>
+      <c r="AV12" s="187"/>
+      <c r="AW12" s="188"/>
+      <c r="AX12" s="186" t="s">
         <v>68</v>
       </c>
-      <c r="AY12" s="181"/>
-      <c r="AZ12" s="181"/>
-      <c r="BA12" s="181"/>
-      <c r="BB12" s="181"/>
-      <c r="BC12" s="181"/>
-      <c r="BD12" s="182"/>
-      <c r="BE12" s="180" t="s">
+      <c r="AY12" s="187"/>
+      <c r="AZ12" s="187"/>
+      <c r="BA12" s="187"/>
+      <c r="BB12" s="187"/>
+      <c r="BC12" s="187"/>
+      <c r="BD12" s="188"/>
+      <c r="BE12" s="186" t="s">
         <v>69</v>
       </c>
-      <c r="BF12" s="181"/>
-      <c r="BG12" s="181"/>
-      <c r="BH12" s="181"/>
-      <c r="BI12" s="181"/>
-      <c r="BJ12" s="181"/>
-      <c r="BK12" s="182"/>
-      <c r="BL12" s="180" t="s">
+      <c r="BF12" s="187"/>
+      <c r="BG12" s="187"/>
+      <c r="BH12" s="187"/>
+      <c r="BI12" s="187"/>
+      <c r="BJ12" s="187"/>
+      <c r="BK12" s="188"/>
+      <c r="BL12" s="186" t="s">
         <v>70</v>
       </c>
-      <c r="BM12" s="181"/>
-      <c r="BN12" s="181"/>
-      <c r="BO12" s="181"/>
-      <c r="BP12" s="181"/>
-      <c r="BQ12" s="181"/>
-      <c r="BR12" s="182"/>
-      <c r="BS12" s="180" t="s">
+      <c r="BM12" s="187"/>
+      <c r="BN12" s="187"/>
+      <c r="BO12" s="187"/>
+      <c r="BP12" s="187"/>
+      <c r="BQ12" s="187"/>
+      <c r="BR12" s="188"/>
+      <c r="BS12" s="186" t="s">
         <v>71</v>
       </c>
-      <c r="BT12" s="181"/>
-      <c r="BU12" s="181"/>
-      <c r="BV12" s="181"/>
-      <c r="BW12" s="181"/>
-      <c r="BX12" s="181"/>
-      <c r="BY12" s="182"/>
-      <c r="BZ12" s="180" t="s">
+      <c r="BT12" s="187"/>
+      <c r="BU12" s="187"/>
+      <c r="BV12" s="187"/>
+      <c r="BW12" s="187"/>
+      <c r="BX12" s="187"/>
+      <c r="BY12" s="188"/>
+      <c r="BZ12" s="186" t="s">
         <v>72</v>
       </c>
-      <c r="CA12" s="181"/>
-      <c r="CB12" s="181"/>
-      <c r="CC12" s="181"/>
-      <c r="CD12" s="181"/>
-      <c r="CE12" s="181"/>
-      <c r="CF12" s="182"/>
-      <c r="CG12" s="180" t="s">
+      <c r="CA12" s="187"/>
+      <c r="CB12" s="187"/>
+      <c r="CC12" s="187"/>
+      <c r="CD12" s="187"/>
+      <c r="CE12" s="187"/>
+      <c r="CF12" s="188"/>
+      <c r="CG12" s="186" t="s">
         <v>73</v>
       </c>
-      <c r="CH12" s="181"/>
-      <c r="CI12" s="181"/>
-      <c r="CJ12" s="181"/>
-      <c r="CK12" s="181"/>
-      <c r="CL12" s="181"/>
-      <c r="CM12" s="182"/>
-      <c r="CN12" s="180" t="s">
+      <c r="CH12" s="187"/>
+      <c r="CI12" s="187"/>
+      <c r="CJ12" s="187"/>
+      <c r="CK12" s="187"/>
+      <c r="CL12" s="187"/>
+      <c r="CM12" s="188"/>
+      <c r="CN12" s="186" t="s">
         <v>74</v>
       </c>
-      <c r="CO12" s="181"/>
-      <c r="CP12" s="181"/>
-      <c r="CQ12" s="181"/>
-      <c r="CR12" s="181"/>
-      <c r="CS12" s="181"/>
-      <c r="CT12" s="182"/>
-      <c r="CU12" s="180" t="s">
+      <c r="CO12" s="187"/>
+      <c r="CP12" s="187"/>
+      <c r="CQ12" s="187"/>
+      <c r="CR12" s="187"/>
+      <c r="CS12" s="187"/>
+      <c r="CT12" s="188"/>
+      <c r="CU12" s="186" t="s">
         <v>75</v>
       </c>
-      <c r="CV12" s="181"/>
-      <c r="CW12" s="181"/>
-      <c r="CX12" s="181"/>
-      <c r="CY12" s="181"/>
-      <c r="CZ12" s="181"/>
-      <c r="DA12" s="182"/>
-      <c r="DB12" s="180" t="s">
+      <c r="CV12" s="187"/>
+      <c r="CW12" s="187"/>
+      <c r="CX12" s="187"/>
+      <c r="CY12" s="187"/>
+      <c r="CZ12" s="187"/>
+      <c r="DA12" s="188"/>
+      <c r="DB12" s="186" t="s">
         <v>76</v>
       </c>
-      <c r="DC12" s="181"/>
-      <c r="DD12" s="181"/>
-      <c r="DE12" s="181"/>
-      <c r="DF12" s="181"/>
-      <c r="DG12" s="181"/>
-      <c r="DH12" s="182"/>
+      <c r="DC12" s="187"/>
+      <c r="DD12" s="187"/>
+      <c r="DE12" s="187"/>
+      <c r="DF12" s="187"/>
+      <c r="DG12" s="187"/>
+      <c r="DH12" s="188"/>
       <c r="DI12" s="183" t="s">
         <v>77</v>
       </c>
@@ -17593,8 +18504,8 @@
     </row>
     <row r="13" spans="2:118" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B13" s="17"/>
-      <c r="C13" s="187"/>
-      <c r="D13" s="187"/>
+      <c r="C13" s="190"/>
+      <c r="D13" s="190"/>
       <c r="E13" s="22">
         <v>7</v>
       </c>
@@ -17940,7 +18851,7 @@
     </row>
     <row r="14" spans="2:118" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B14" s="17"/>
-      <c r="C14" s="186" t="s">
+      <c r="C14" s="189" t="s">
         <v>78</v>
       </c>
       <c r="D14" s="24" t="s">
@@ -18063,7 +18974,7 @@
     </row>
     <row r="15" spans="2:118" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B15" s="32"/>
-      <c r="C15" s="187"/>
+      <c r="C15" s="190"/>
       <c r="D15" s="33" t="s">
         <v>84</v>
       </c>
@@ -18184,7 +19095,7 @@
     </row>
     <row r="16" spans="2:118" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B16" s="32"/>
-      <c r="C16" s="187"/>
+      <c r="C16" s="190"/>
       <c r="D16" s="33" t="s">
         <v>85</v>
       </c>
@@ -18305,7 +19216,7 @@
     </row>
     <row r="17" spans="2:118" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B17" s="32"/>
-      <c r="C17" s="187"/>
+      <c r="C17" s="190"/>
       <c r="D17" s="33" t="s">
         <v>86</v>
       </c>
@@ -18426,7 +19337,7 @@
     </row>
     <row r="18" spans="2:118" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B18" s="32"/>
-      <c r="C18" s="187"/>
+      <c r="C18" s="190"/>
       <c r="D18" s="33" t="s">
         <v>87</v>
       </c>
@@ -18547,7 +19458,7 @@
     </row>
     <row r="19" spans="2:118" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B19" s="32"/>
-      <c r="C19" s="187"/>
+      <c r="C19" s="190"/>
       <c r="D19" s="33" t="s">
         <v>88</v>
       </c>
@@ -18668,7 +19579,7 @@
     </row>
     <row r="20" spans="2:118" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="17"/>
-      <c r="C20" s="188"/>
+      <c r="C20" s="191"/>
       <c r="D20" s="24" t="s">
         <v>89</v>
       </c>
@@ -42827,7 +43738,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="D12:D13"/>
     <mergeCell ref="E12:G12"/>
     <mergeCell ref="H12:N12"/>
     <mergeCell ref="O12:U12"/>
@@ -42847,6 +43757,7 @@
     <mergeCell ref="AX12:BD12"/>
     <mergeCell ref="BE12:BK12"/>
     <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>